<commit_message>
fix(calculators): ignore the burnt fraction for crops with no burning factor
Table A.2.1.1 gives no fraction of residue remaining at burning (Sc, n/a)
for cotton, hops and grape vines, tubers and roots, forage crops and other
annual/perennial crops, so 6.4 field burning is always zero for them. 6.1
still subtracted the farmer's burnt fraction (Fc) from the residue returned
to the soil, so entering a burn lowered total emissions (and could make Mc
negative for tubers and roots, where FFODc is already 1). Treat Fc as 0 in
Mc when the crop has no Sc, matching v3, which hard-coded Fc = 0 for cotton
and vineyards. Updates the 6.1 and 6.3 test workbooks to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/6.1-crop-residues.xlsx
+++ b/packages/calculators/src/modules/test/6.1-crop-residues.xlsx
@@ -1202,7 +1202,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="O5">
-        <f t="shared" ref="O5:O14" si="5">IF(ISBLANK(A5),"", (G5*H5*(1 - D5 - F5) * J5*L5)+(G5*H5*I5*J5*N5))</f>
+        <f t="shared" ref="O5:O14" si="5">IF(ISBLANK(A5),"", (G5*H5*(1 - IF(ISNUMBER(VLOOKUP($B5, $S$22:$AA$39, 8, FALSE)), D5, 0) - F5) * J5*L5)+(G5*H5*I5*J5*N5))</f>
         <v>0.35750000000000004</v>
       </c>
       <c r="P5">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="O9">
         <f t="shared" si="5"/>
-        <v>3.5700000000000065E-2</v>
+        <v>0.5117</v>
       </c>
       <c r="P9">
         <f t="shared" si="6"/>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="Q9">
         <f t="shared" si="7"/>
-        <v>3.3629400000000059E-7</v>
+        <v>4.820214000000001e-06</v>
       </c>
       <c r="S9" s="2"/>
       <c r="T9" s="2"/>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="O10">
         <f t="shared" si="5"/>
-        <v>-0.21675000000000011</v>
+        <v>0.54825</v>
       </c>
       <c r="P10">
         <f t="shared" si="6"/>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="Q10">
         <f t="shared" si="7"/>
-        <v>-2.0417850000000012E-6</v>
+        <v>5.1645150000000005e-06</v>
       </c>
       <c r="S10" t="s">
         <v>2</v>
@@ -1580,7 +1580,7 @@
       </c>
       <c r="O11">
         <f t="shared" si="5"/>
-        <v>27.36</v>
+        <v>35.568</v>
       </c>
       <c r="P11">
         <f t="shared" si="6"/>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="Q11">
         <f t="shared" si="7"/>
-        <v>2.5773119999999999E-4</v>
+        <v>0.00033505055999999997</v>
       </c>
       <c r="S11" s="2"/>
       <c r="T11" s="2"/>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="O12">
         <f t="shared" si="5"/>
-        <v>9.4247999999999994</v>
+        <v>13.464</v>
       </c>
       <c r="P12">
         <f t="shared" si="6"/>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="Q12">
         <f t="shared" si="7"/>
-        <v>8.8781615999999994E-5</v>
+        <v>0.00012683088</v>
       </c>
       <c r="S12" s="2" t="s">
         <v>6</v>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="O13">
         <f t="shared" si="5"/>
-        <v>6.5799359999999982</v>
+        <v>10.400543999999998</v>
       </c>
       <c r="P13">
         <f t="shared" si="6"/>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="Q13">
         <f t="shared" si="7"/>
-        <v>6.1982997119999989E-5</v>
+        <v>9.797312447999999e-05</v>
       </c>
       <c r="S13" t="s">
         <v>7</v>
@@ -1889,7 +1889,7 @@
         <v>0.01</v>
       </c>
       <c r="O17">
-        <f>IF(ISBLANK(A17),"", (G17*H17*(1 - D17 - F17) * J17*L17)+(G17*H17*I17*J17*N17))</f>
+        <f>IF(ISBLANK(A17),"", (G17*H17*(1 - IF(ISNUMBER(VLOOKUP($B17, $S$22:$AA$39, 8, FALSE)), D17, 0) - F17) * J17*L17)+(G17*H17*I17*J17*N17))</f>
         <v>13.3064</v>
       </c>
       <c r="P17">
@@ -1953,7 +1953,7 @@
         <v>0.01</v>
       </c>
       <c r="O18">
-        <f>IF(ISBLANK(A18),"", (G18*H18*(1 - D18 - F18) * J18*L18)+(G18*H18*I18*J18*N18))</f>
+        <f>IF(ISBLANK(A18),"", (G18*H18*(1 - IF(ISNUMBER(VLOOKUP($B18, $S$22:$AA$39, 8, FALSE)), D18, 0) - F18) * J18*L18)+(G18*H18*I18*J18*N18))</f>
         <v>28.511118000000003</v>
       </c>
       <c r="P18">
@@ -2019,8 +2019,8 @@
         <v>0</v>
       </c>
       <c r="O19">
-        <f>IF(ISBLANK(A19),"", (G19*H19*(1 - D19 - F19) * J19*L19)+(G19*H19*I19*J19*N19))</f>
-        <v>11.193599999999998</v>
+        <f>IF(ISBLANK(A19),"", (G19*H19*(1 - IF(ISNUMBER(VLOOKUP($B19, $S$22:$AA$39, 8, FALSE)), D19, 0) - F19) * J19*L19)+(G19*H19*I19*J19*N19))</f>
+        <v>16.896</v>
       </c>
       <c r="P19">
         <f>IF(ISBLANK(A19),"",VLOOKUP(A19,$S$14:$T$30,2,FALSE))</f>
@@ -2028,7 +2028,7 @@
       </c>
       <c r="Q19">
         <f>IF(ISBLANK(A19), "", O19*P19*$T$10/1000)</f>
-        <v>1.0544371199999999E-4</v>
+        <v>0.00015916032</v>
       </c>
       <c r="S19" s="2"/>
       <c r="T19" s="2"/>
@@ -2085,8 +2085,8 @@
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="O20">
-        <f>IF(ISBLANK(A20),"", (G20*H20*(1 - D20 - F20) * J20*L20)+(G20*H20*I20*J20*N20))</f>
-        <v>16.073499999999996</v>
+        <f>IF(ISBLANK(A20),"", (G20*H20*(1 - IF(ISNUMBER(VLOOKUP($B20, $S$22:$AA$39, 8, FALSE)), D20, 0) - F20) * J20*L20)+(G20*H20*I20*J20*N20))</f>
+        <v>21.1735</v>
       </c>
       <c r="P20">
         <f>IF(ISBLANK(A20),"",VLOOKUP(A20,$S$14:$T$30,2,FALSE))</f>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="Q20">
         <f>IF(ISBLANK(A20), "", O20*P20*$T$10/1000)</f>
-        <v>1.5141236999999995E-4</v>
+        <v>0.00019945437000000002</v>
       </c>
       <c r="S20" s="2" t="s">
         <v>15</v>

</xml_diff>